<commit_message>
Sync latest UI and cleanup changes
</commit_message>
<xml_diff>
--- a/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
+++ b/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tushargarg/Downloads/expense_register-main 2/assets/samples/sample_budget_uploads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3616A984-C14E-4741-8487-86F00CE00CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
   <si>
     <t>Department</t>
   </si>
@@ -134,14 +139,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -168,13 +168,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -464,23 +472,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -503,7 +507,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -517,7 +521,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -526,7 +530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -549,7 +553,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -572,7 +576,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -595,7 +599,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -618,7 +622,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -641,7 +645,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -664,7 +668,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -687,7 +691,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -710,7 +714,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -733,7 +737,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -756,7 +760,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -780,8 +784,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: Expense reassignment visibility and approval controls
- Remove others option from expense list request filter
- Remove action history section from expense review page
- Add confirmation dialogs for approve, reject, and reassign actions
- Hide sidebar for temporary reassigned approvers
- Fix expense list visibility for reassigned non-head approvers
- Allow pending_approvals scope for users with reassigned tasks
- Add hasPendingAssignmentForUser() helper to detect reassignments
</commit_message>
<xml_diff>
--- a/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
+++ b/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tushargarg/Downloads/expense_register-main 2/assets/samples/sample_budget_uploads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/expense_register/assets/samples/sample_budget_uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3616A984-C14E-4741-8487-86F00CE00CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5067FC1B-E55C-D445-8190-12CFB97849BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t>Department</t>
   </si>
@@ -55,9 +55,6 @@
     <t>INR</t>
   </si>
   <si>
-    <t>IT travel allocation Q1</t>
-  </si>
-  <si>
     <t>FINANCE</t>
   </si>
   <si>
@@ -134,17 +131,29 @@
   </si>
   <si>
     <t>Sales team office supplies</t>
+  </si>
+  <si>
+    <t>PARKING</t>
+  </si>
+  <si>
+    <t>IT Parking allocation Q2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,8 +176,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,37 +521,37 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
+      <c r="B2" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="E2">
-        <v>300000</v>
+        <v>20000</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
-        <v>11</v>
+      <c r="G2" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3">
+        <v>2026</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3">
-        <v>2026</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
       </c>
       <c r="E3">
         <v>180000</v>
@@ -550,15 +560,15 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
       </c>
       <c r="C4">
         <v>2026</v>
@@ -573,21 +583,21 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5">
+        <v>2026</v>
+      </c>
+      <c r="D5" t="s">
         <v>20</v>
-      </c>
-      <c r="C5">
-        <v>2026</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
       </c>
       <c r="E5">
         <v>95000</v>
@@ -596,12 +606,12 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -610,7 +620,7 @@
         <v>2026</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>160000</v>
@@ -619,21 +629,21 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
-      </c>
-      <c r="C7">
-        <v>2026</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
       <c r="E7">
         <v>300000</v>
@@ -642,15 +652,15 @@
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
       </c>
       <c r="C8">
         <v>2026</v>
@@ -665,7 +675,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -673,13 +683,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>2026</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>210000</v>
@@ -688,21 +698,21 @@
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10">
         <v>2026</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10">
         <v>500000</v>
@@ -711,21 +721,21 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
       <c r="C11">
         <v>2026</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11">
         <v>140000</v>
@@ -734,12 +744,12 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -748,7 +758,7 @@
         <v>2026</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12">
         <v>110000</v>
@@ -757,15 +767,15 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13">
         <v>2026</v>
@@ -780,7 +790,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync latest project updates
</commit_message>
<xml_diff>
--- a/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
+++ b/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tushargarg/Downloads/expense_register-main 2/assets/samples/sample_budget_uploads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/expense_register/assets/samples/sample_budget_uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3616A984-C14E-4741-8487-86F00CE00CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5067FC1B-E55C-D445-8190-12CFB97849BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t>Department</t>
   </si>
@@ -55,9 +55,6 @@
     <t>INR</t>
   </si>
   <si>
-    <t>IT travel allocation Q1</t>
-  </si>
-  <si>
     <t>FINANCE</t>
   </si>
   <si>
@@ -134,17 +131,29 @@
   </si>
   <si>
     <t>Sales team office supplies</t>
+  </si>
+  <si>
+    <t>PARKING</t>
+  </si>
+  <si>
+    <t>IT Parking allocation Q2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,8 +176,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,37 +521,37 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
+      <c r="B2" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="E2">
-        <v>300000</v>
+        <v>20000</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
-        <v>11</v>
+      <c r="G2" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3">
+        <v>2026</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3">
-        <v>2026</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
       </c>
       <c r="E3">
         <v>180000</v>
@@ -550,15 +560,15 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
       </c>
       <c r="C4">
         <v>2026</v>
@@ -573,21 +583,21 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5">
+        <v>2026</v>
+      </c>
+      <c r="D5" t="s">
         <v>20</v>
-      </c>
-      <c r="C5">
-        <v>2026</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
       </c>
       <c r="E5">
         <v>95000</v>
@@ -596,12 +606,12 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -610,7 +620,7 @@
         <v>2026</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>160000</v>
@@ -619,21 +629,21 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
-      </c>
-      <c r="C7">
-        <v>2026</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
       <c r="E7">
         <v>300000</v>
@@ -642,15 +652,15 @@
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
       </c>
       <c r="C8">
         <v>2026</v>
@@ -665,7 +675,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -673,13 +683,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>2026</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>210000</v>
@@ -688,21 +698,21 @@
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10">
         <v>2026</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10">
         <v>500000</v>
@@ -711,21 +721,21 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
       <c r="C11">
         <v>2026</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11">
         <v>140000</v>
@@ -734,12 +744,12 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -748,7 +758,7 @@
         <v>2026</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12">
         <v>110000</v>
@@ -757,15 +767,15 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13">
         <v>2026</v>
@@ -780,7 +790,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update controllers, models, views, and schema for expense management and authentication
</commit_message>
<xml_diff>
--- a/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
+++ b/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/expense_register/assets/samples/sample_budget_uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5067FC1B-E55C-D445-8190-12CFB97849BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C351CF4A-9D6D-8D4E-B652-907A0B13FB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Department</t>
   </si>
@@ -46,9 +46,6 @@
     <t>IT</t>
   </si>
   <si>
-    <t>TRAVEL</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -76,33 +73,12 @@
     <t>HR hiring allocation Q1</t>
   </si>
   <si>
-    <t>MARKETING</t>
-  </si>
-  <si>
-    <t>OFFICE SUPPLIES</t>
-  </si>
-  <si>
     <t>Q3</t>
   </si>
   <si>
-    <t>Marketing stationery and supplies</t>
-  </si>
-  <si>
-    <t>SALES</t>
-  </si>
-  <si>
-    <t>Sales travel and client visits</t>
-  </si>
-  <si>
-    <t>RENT AND UTILITIES</t>
-  </si>
-  <si>
     <t>Q4</t>
   </si>
   <si>
-    <t>Operations overhead allocation</t>
-  </si>
-  <si>
     <t>ADMIN</t>
   </si>
   <si>
@@ -125,12 +101,6 @@
   </si>
   <si>
     <t>HR onboarding and recruiting</t>
-  </si>
-  <si>
-    <t>Campaign travel allocation</t>
-  </si>
-  <si>
-    <t>Sales team office supplies</t>
   </si>
   <si>
     <t>PARKING</t>
@@ -483,7 +453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -522,88 +492,88 @@
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>20000</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
       <c r="C3">
         <v>2026</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3">
         <v>180000</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
       </c>
       <c r="C4">
         <v>2026</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4">
         <v>120000</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>2026</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>95000</v>
+        <v>70000</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
         <v>21</v>
@@ -611,22 +581,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
       </c>
       <c r="C6">
         <v>2026</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6">
-        <v>160000</v>
+        <v>210000</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" t="s">
         <v>23</v>
@@ -634,7 +604,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>24</v>
@@ -643,154 +613,39 @@
         <v>2026</v>
       </c>
       <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7">
+        <v>500000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
         <v>25</v>
-      </c>
-      <c r="E7">
-        <v>300000</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>2026</v>
       </c>
       <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8">
+        <v>140000</v>
+      </c>
+      <c r="F8" t="s">
         <v>9</v>
       </c>
-      <c r="E8">
-        <v>70000</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
       <c r="G8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9">
-        <v>2026</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9">
-        <v>210000</v>
-      </c>
-      <c r="F9" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10">
-        <v>2026</v>
-      </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10">
-        <v>500000</v>
-      </c>
-      <c r="F10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11">
-        <v>2026</v>
-      </c>
-      <c r="D11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11">
-        <v>140000</v>
-      </c>
-      <c r="F11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12">
-        <v>2026</v>
-      </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12">
-        <v>110000</v>
-      </c>
-      <c r="F12" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13">
-        <v>2026</v>
-      </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13">
-        <v>60000</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: latest changes before Bitbucket push (2026-04-26)
</commit_message>
<xml_diff>
--- a/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
+++ b/assets/samples/sample_budget_uploads/budget_upload_all_correct.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/expense_register/assets/samples/sample_budget_uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5067FC1B-E55C-D445-8190-12CFB97849BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C351CF4A-9D6D-8D4E-B652-907A0B13FB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Department</t>
   </si>
@@ -46,9 +46,6 @@
     <t>IT</t>
   </si>
   <si>
-    <t>TRAVEL</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -76,33 +73,12 @@
     <t>HR hiring allocation Q1</t>
   </si>
   <si>
-    <t>MARKETING</t>
-  </si>
-  <si>
-    <t>OFFICE SUPPLIES</t>
-  </si>
-  <si>
     <t>Q3</t>
   </si>
   <si>
-    <t>Marketing stationery and supplies</t>
-  </si>
-  <si>
-    <t>SALES</t>
-  </si>
-  <si>
-    <t>Sales travel and client visits</t>
-  </si>
-  <si>
-    <t>RENT AND UTILITIES</t>
-  </si>
-  <si>
     <t>Q4</t>
   </si>
   <si>
-    <t>Operations overhead allocation</t>
-  </si>
-  <si>
     <t>ADMIN</t>
   </si>
   <si>
@@ -125,12 +101,6 @@
   </si>
   <si>
     <t>HR onboarding and recruiting</t>
-  </si>
-  <si>
-    <t>Campaign travel allocation</t>
-  </si>
-  <si>
-    <t>Sales team office supplies</t>
   </si>
   <si>
     <t>PARKING</t>
@@ -483,7 +453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -522,88 +492,88 @@
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>20000</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
       <c r="C3">
         <v>2026</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3">
         <v>180000</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
       </c>
       <c r="C4">
         <v>2026</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4">
         <v>120000</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>2026</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>95000</v>
+        <v>70000</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
         <v>21</v>
@@ -611,22 +581,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
       </c>
       <c r="C6">
         <v>2026</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6">
-        <v>160000</v>
+        <v>210000</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" t="s">
         <v>23</v>
@@ -634,7 +604,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>24</v>
@@ -643,154 +613,39 @@
         <v>2026</v>
       </c>
       <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7">
+        <v>500000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
         <v>25</v>
-      </c>
-      <c r="E7">
-        <v>300000</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>2026</v>
       </c>
       <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8">
+        <v>140000</v>
+      </c>
+      <c r="F8" t="s">
         <v>9</v>
       </c>
-      <c r="E8">
-        <v>70000</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
       <c r="G8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9">
-        <v>2026</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9">
-        <v>210000</v>
-      </c>
-      <c r="F9" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10">
-        <v>2026</v>
-      </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10">
-        <v>500000</v>
-      </c>
-      <c r="F10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11">
-        <v>2026</v>
-      </c>
-      <c r="D11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11">
-        <v>140000</v>
-      </c>
-      <c r="F11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12">
-        <v>2026</v>
-      </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12">
-        <v>110000</v>
-      </c>
-      <c r="F12" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13">
-        <v>2026</v>
-      </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13">
-        <v>60000</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>